<commit_message>
docs: actualizacion matriz de casos
</commit_message>
<xml_diff>
--- a/Matriz_de_casos_.xlsx
+++ b/Matriz_de_casos_.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Casos de prueba" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="68">
   <si>
     <t xml:space="preserve"> QA Test: https://www.saucedemo.com/</t>
   </si>
@@ -207,7 +207,7 @@
     <t>009_compra_producto_exitoso_carrito</t>
   </si>
   <si>
-    <t>validar que el usuario pueda realizar el pedito de compra.</t>
+    <t>validar que el usuario pueda realizar el pedido de compra.</t>
   </si>
   <si>
     <t>1. ingresar a la pagína https://www.saucedemo.com/ 
@@ -254,10 +254,26 @@
     <t>El usuario debe ver los productos ordenados de la A-Z</t>
   </si>
   <si>
-    <t>011_ordenar_productos_por_precio_mayor_menor</t>
-  </si>
-  <si>
-    <t>validar que el usuario pueda visualizar los productos ordenados por precio de mator a menor</t>
+    <t>012_ordenar_productos_por_precio_mayor_menor</t>
+  </si>
+  <si>
+    <t>validar que el usuario pueda visualizar los productos ordenados por precio de mayor a menor</t>
+  </si>
+  <si>
+    <t>1. ingresar a la pagína https://www.saucedemo.com/ 
+2. ingresar el usuario validos.
+3. ingresar el password validos.
+4. Seleccionar un producto.
+5. En los filtros seleccionar la opcion 'Price (hight o low)'</t>
+  </si>
+  <si>
+    <t>El usuario debe ver los productos ordenados por precio de mayor a menor</t>
+  </si>
+  <si>
+    <t>013_ordenar_productos_por_precio_menor_meyor</t>
+  </si>
+  <si>
+    <t>validar que el usuario pueda visualizar los productos ordenados por precio menor a mayor</t>
   </si>
   <si>
     <t>1. ingresar a la pagína https://www.saucedemo.com/ 
@@ -267,7 +283,7 @@
 5. En los filtros seleccionar la opcion 'Price (low to high)'</t>
   </si>
   <si>
-    <t>El usuario debe ver los productos ordenados por precio de mayor a menor</t>
+    <t>El usuario debe ver los productos ordenados por precio de menor a mayor</t>
   </si>
 </sst>
 </file>
@@ -280,7 +296,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -297,13 +313,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -448,7 +457,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -469,12 +478,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -602,12 +605,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -821,67 +818,70 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -896,46 +896,49 @@
     <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -944,10 +947,10 @@
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -956,17 +959,11 @@
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -984,9 +981,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1013,12 +1007,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1342,7 +1330,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.5714285714286" style="1" customWidth="1"/>
@@ -1398,325 +1386,357 @@
       <c r="G2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
     </row>
     <row r="3" ht="75" spans="1:18">
-      <c r="A3" s="9">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" ht="75" spans="1:18">
-      <c r="A4" s="9">
+      <c r="A4" s="8">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="75" spans="1:18">
-      <c r="A5" s="9">
+      <c r="A5" s="8">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" ht="90" spans="1:18">
-      <c r="A6" s="9">
+      <c r="A6" s="8">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" ht="90" spans="1:18">
-      <c r="A7" s="9">
+      <c r="A7" s="8">
         <v>5</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" ht="75" spans="1:18">
-      <c r="A8" s="9">
+      <c r="A8" s="8">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" ht="90" spans="1:18">
-      <c r="A9" s="9">
+      <c r="A9" s="8">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" ht="90" spans="1:18">
-      <c r="A10" s="9">
+      <c r="A10" s="8">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" ht="135" spans="1:18">
-      <c r="A11" s="17">
+      <c r="A11" s="8">
         <v>9</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" ht="105" spans="1:18">
-      <c r="A12" s="17">
+      <c r="A12" s="8">
         <v>10</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H12" s="18"/>
+      <c r="H12" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" ht="105" spans="1:18">
-      <c r="A13" s="17">
+      <c r="A13" s="8">
         <v>11</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H13" s="18"/>
+      <c r="H13" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" ht="105" spans="1:18">
-      <c r="A14" s="17">
-        <v>11</v>
-      </c>
-      <c r="B14" s="10" t="s">
+      <c r="A14" s="8">
+        <v>12</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="18"/>
+      <c r="H14" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="105" spans="1:18">
+      <c r="A15" s="8">
+        <v>13</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>